<commit_message>
feat(web): expand workbook rule rendering
</commit_message>
<xml_diff>
--- a/testdata/compatibility/feature-rich.xlsx
+++ b/testdata/compatibility/feature-rich.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Category</t>
   </si>
@@ -46,22 +46,73 @@
     <t>Choice</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Whole</t>
+  </si>
+  <si>
+    <t>Range choice</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Scale</t>
+  </si>
+  <si>
+    <t>Bar</t>
+  </si>
+  <si>
+    <t>Duplicate</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Allowed values</t>
+  </si>
+  <si>
     <t>Alpha</t>
   </si>
   <si>
     <t>A</t>
   </si>
   <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Alpha item</t>
+  </si>
+  <si>
+    <t>Repeat</t>
+  </si>
+  <si>
     <t>Beta</t>
   </si>
   <si>
     <t>B</t>
   </si>
   <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Beta item</t>
+  </si>
+  <si>
+    <t>Unique</t>
+  </si>
+  <si>
     <t>Gamma</t>
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>Alpha note</t>
   </si>
   <si>
     <t>Merged heading</t>
@@ -362,13 +413,13 @@
 <xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -392,13 +443,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
@@ -703,10 +754,40 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1">
         <v>1250.5</v>
@@ -715,18 +796,43 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F2" t="str">
         <f>'[external-source.xlsx]Sheet1'!$A$1</f>
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>15</v>
+      </c>
+      <c r="L2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2">
+        <v>45292</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
         <v>845.25</v>
@@ -735,12 +841,42 @@
         <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3">
+        <v>50</v>
+      </c>
+      <c r="K3">
+        <v>45</v>
+      </c>
+      <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3">
+        <v>45474</v>
+      </c>
+      <c r="N3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1">
         <v>420.75</v>
@@ -749,7 +885,37 @@
         <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>75</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4">
+        <v>90</v>
+      </c>
+      <c r="K4">
+        <v>85</v>
+      </c>
+      <c r="L4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4">
+        <v>45657</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -759,7 +925,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -771,9 +937,52 @@
       <formula>15</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <conditionalFormatting sqref="I2:I4">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Alpha">
+      <formula>NOT(ISERROR(SEARCH("Alpha",I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J4">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K4">
+    <cfRule type="dataBar" priority="4">
+      <dataBar showValue="true">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L4">
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+  </conditionalFormatting>
+  <dataValidations count="5">
     <dataValidation allowBlank="true" sqref="D2:D10" type="list">
       <formula1>"A,B,C"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="The value must be a whole number from 1 through 100." errorStyle="stop" errorTitle="Invalid number" operator="between" prompt="Enter a whole number from 1 through 100." promptTitle="Whole number" showErrorMessage="true" showInputMessage="true" sqref="G2:G10" type="whole">
+      <formula1>1</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="H2:H10" type="list">
+      <formula1>$N$2:$N$4</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Use no more than 12 characters." errorStyle="warning" errorTitle="Long text" showErrorMessage="true" sqref="I2:I10" type="custom">
+      <formula1>LEN(I2)&lt;=12</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="between" sqref="M2:M10" type="date">
+      <formula1>45292</formula1>
+      <formula2>45657</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>